<commit_message>
Timesheet Project Local Deployment 14/08/2026
</commit_message>
<xml_diff>
--- a/Timesheet-Project/Timesheet 3/Buhle/Buhle_Mukhuba_April_FinalWeek.xlsx
+++ b/Timesheet-Project/Timesheet 3/Buhle/Buhle_Mukhuba_April_FinalWeek.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30023"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\sc_LwazisileMhlambi_2026\Timesheet-Project\Timesheet 3\Buhle\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://northerndata-my.sharepoint.com/personal/buhle_mukhuba_sambeconsulting_com/Documents/Documents/Timesheets/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="145" documentId="8_{DD65C2EA-B99D-4478-A49F-4E4F7E176690}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{48A32F68-EF15-4545-8712-DC6F9622A224}"/>
@@ -656,7 +656,7 @@
     <numFmt numFmtId="164" formatCode="[h]:mm"/>
     <numFmt numFmtId="165" formatCode="h:mm;@"/>
   </numFmts>
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="19">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1356,118 +1356,6 @@
   </cellStyles>
   <dxfs count="23">
     <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <font>
         <b val="0"/>
         <i val="0"/>
@@ -1608,6 +1496,118 @@
         <scheme val="none"/>
       </font>
     </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="Invisible" pivot="0" table="0" count="0" xr9:uid="{6758C6CA-2356-4535-9D9D-86230C423211}"/>
@@ -1673,26 +1673,26 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2E876225-7964-4082-91F1-C6221C464408}" name="WorkType" displayName="WorkType" ref="H2:H76" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2E876225-7964-4082-91F1-C6221C464408}" name="WorkType" displayName="WorkType" ref="H2:H76" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5">
   <autoFilter ref="H2:H76" xr:uid="{2E876225-7964-4082-91F1-C6221C464408}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="H3:H76">
     <sortCondition ref="H64:H76"/>
   </sortState>
   <tableColumns count="1">
-    <tableColumn id="2" xr3:uid="{234A6588-4DEA-4067-9367-AEAFE02CA40D}" name="Resource" dataDxfId="20"/>
+    <tableColumn id="2" xr3:uid="{234A6588-4DEA-4067-9367-AEAFE02CA40D}" name="Resource" dataDxfId="4"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{B149CFBE-03DA-4A5C-8F86-52A53133C863}" name="ProjectTable" displayName="ProjectTable" ref="F2:F40" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18" tableBorderDxfId="17">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{B149CFBE-03DA-4A5C-8F86-52A53133C863}" name="ProjectTable" displayName="ProjectTable" ref="F2:F40" totalsRowShown="0" headerRowDxfId="3" dataDxfId="2" tableBorderDxfId="1">
   <autoFilter ref="F2:F40" xr:uid="{B149CFBE-03DA-4A5C-8F86-52A53133C863}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="F3:F19">
     <sortCondition ref="F2:F19"/>
   </sortState>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{D9788319-59C4-447A-9364-6F4EF6730453}" name="Description" dataDxfId="16"/>
+    <tableColumn id="1" xr3:uid="{D9788319-59C4-447A-9364-6F4EF6730453}" name="Description" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1969,18 +1969,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B63D3D5-6C83-45F2-B2A7-43EE15BF1EF3}">
   <dimension ref="A5:J158"/>
-  <sheetFormatPr defaultColWidth="8.69921875" defaultRowHeight="12.6" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.75" defaultRowHeight="12.6"/>
   <cols>
     <col min="1" max="1" width="12" style="21" customWidth="1"/>
-    <col min="2" max="2" width="13.09765625" style="21" customWidth="1"/>
-    <col min="3" max="3" width="16.19921875" style="21" customWidth="1"/>
+    <col min="2" max="2" width="13.125" style="21" customWidth="1"/>
+    <col min="3" max="3" width="16.25" style="21" customWidth="1"/>
     <col min="4" max="5" width="20" style="21" customWidth="1"/>
-    <col min="6" max="6" width="23.09765625" style="21" customWidth="1"/>
+    <col min="6" max="6" width="23.125" style="21" customWidth="1"/>
     <col min="7" max="7" width="34" style="21" customWidth="1"/>
-    <col min="8" max="16384" width="8.69921875" style="21"/>
+    <col min="8" max="16384" width="8.75" style="21"/>
   </cols>
   <sheetData>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:10">
       <c r="A5" s="34" t="s">
         <v>0</v>
       </c>
@@ -1989,7 +1989,7 @@
       </c>
       <c r="H5" s="37"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:10">
       <c r="A6" s="34" t="s">
         <v>2</v>
       </c>
@@ -2001,7 +2001,7 @@
       <c r="H6" s="37"/>
       <c r="J6" s="38"/>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:10">
       <c r="A7" s="34"/>
       <c r="B7" s="42"/>
       <c r="C7" s="34"/>
@@ -2010,7 +2010,7 @@
       <c r="H7" s="37"/>
       <c r="J7" s="38"/>
     </row>
-    <row r="8" spans="1:10" ht="25.2" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:10" ht="25.15">
       <c r="A8" s="22" t="s">
         <v>3</v>
       </c>
@@ -2042,7 +2042,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:10">
       <c r="A9" s="20">
         <v>46113</v>
       </c>
@@ -2073,7 +2073,7 @@
         <v>0.34513888888888888</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:10">
       <c r="A10" s="20">
         <v>46113</v>
       </c>
@@ -2104,7 +2104,7 @@
         <v>0.4548611111111111</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:10">
       <c r="A11" s="20">
         <v>46113</v>
       </c>
@@ -2135,7 +2135,7 @@
         <v>0.48333333333333334</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:10">
       <c r="A12" s="20">
         <v>46113</v>
       </c>
@@ -2166,7 +2166,7 @@
         <v>0.52083333333333337</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:10">
       <c r="A13" s="20">
         <v>46113</v>
       </c>
@@ -2197,7 +2197,7 @@
         <v>0.66319444444444442</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="25.2" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:10" ht="25.15">
       <c r="A14" s="20">
         <v>46113</v>
       </c>
@@ -2228,7 +2228,7 @@
         <v>0.73263888888888884</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:10">
       <c r="A15" s="20">
         <v>46113</v>
       </c>
@@ -2259,7 +2259,7 @@
         <v>0.75347222222222221</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:10">
       <c r="A16" s="20">
         <v>46114</v>
       </c>
@@ -2290,7 +2290,7 @@
         <v>0.33680555555555558</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:10">
       <c r="A17" s="20">
         <v>46114</v>
       </c>
@@ -2321,7 +2321,7 @@
         <v>0.4548611111111111</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:10">
       <c r="A18" s="20">
         <v>46114</v>
       </c>
@@ -2352,7 +2352,7 @@
         <v>0.49375000000000002</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:10">
       <c r="A19" s="20">
         <v>46114</v>
       </c>
@@ -2383,7 +2383,7 @@
         <v>0.53125</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:10">
       <c r="A20" s="20">
         <v>46114</v>
       </c>
@@ -2414,7 +2414,7 @@
         <v>0.66319444444444442</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="25.2" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:10" ht="25.15">
       <c r="A21" s="20">
         <v>46114</v>
       </c>
@@ -2445,7 +2445,7 @@
         <v>0.71597222222222223</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:10">
       <c r="A22" s="43">
         <v>46115</v>
       </c>
@@ -2476,7 +2476,7 @@
         <v>0.66666666666666663</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:10">
       <c r="A23" s="29">
         <v>46116</v>
       </c>
@@ -2495,7 +2495,7 @@
       <c r="I23" s="33"/>
       <c r="J23" s="33"/>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:10">
       <c r="A24" s="29">
         <v>46117</v>
       </c>
@@ -2514,7 +2514,7 @@
       <c r="I24" s="33"/>
       <c r="J24" s="33"/>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:10">
       <c r="A25" s="43">
         <v>46118</v>
       </c>
@@ -2545,7 +2545,7 @@
         <v>0.66666666666666663</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:10">
       <c r="A26" s="20">
         <v>46119</v>
       </c>
@@ -2576,7 +2576,7 @@
         <v>0.34027777777777779</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:10">
       <c r="A27" s="20">
         <v>46119</v>
       </c>
@@ -2607,7 +2607,7 @@
         <v>0.4548611111111111</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:10">
       <c r="A28" s="20">
         <v>46119</v>
       </c>
@@ -2638,7 +2638,7 @@
         <v>0.48541666666666666</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:10">
       <c r="A29" s="20">
         <v>46119</v>
       </c>
@@ -2669,7 +2669,7 @@
         <v>0.52083333333333337</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:10">
       <c r="A30" s="20">
         <v>46119</v>
       </c>
@@ -2700,7 +2700,7 @@
         <v>0.66319444444444442</v>
       </c>
     </row>
-    <row r="31" spans="1:10" ht="25.2" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:10" ht="25.15">
       <c r="A31" s="20">
         <v>46119</v>
       </c>
@@ -2731,7 +2731,7 @@
         <v>0.70486111111111116</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:10">
       <c r="A32" s="20">
         <v>46119</v>
       </c>
@@ -2762,7 +2762,7 @@
         <v>0.72638888888888886</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:10">
       <c r="A33" s="20">
         <v>46120</v>
       </c>
@@ -2793,7 +2793,7 @@
         <v>0.34097222222222223</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:10">
       <c r="A34" s="20">
         <v>46120</v>
       </c>
@@ -2824,7 +2824,7 @@
         <v>0.4548611111111111</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:10">
       <c r="A35" s="20">
         <v>46120</v>
       </c>
@@ -2855,7 +2855,7 @@
         <v>0.4909722222222222</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:10">
       <c r="A36" s="20">
         <v>46120</v>
       </c>
@@ -2886,7 +2886,7 @@
         <v>0.52777777777777779</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:10">
       <c r="A37" s="20">
         <v>46120</v>
       </c>
@@ -2917,7 +2917,7 @@
         <v>0.66319444444444442</v>
       </c>
     </row>
-    <row r="38" spans="1:10" ht="25.2" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:10" ht="25.15">
       <c r="A38" s="20">
         <v>46120</v>
       </c>
@@ -2948,7 +2948,7 @@
         <v>0.68888888888888888</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:10">
       <c r="A39" s="20">
         <v>46120</v>
       </c>
@@ -2979,7 +2979,7 @@
         <v>0.71527777777777779</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:10">
       <c r="A40" s="20">
         <v>46121</v>
       </c>
@@ -3010,7 +3010,7 @@
         <v>0.33402777777777776</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:10">
       <c r="A41" s="20">
         <v>46121</v>
       </c>
@@ -3041,7 +3041,7 @@
         <v>0.39930555555555558</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:10">
       <c r="A42" s="20">
         <v>46121</v>
       </c>
@@ -3072,7 +3072,7 @@
         <v>0.4548611111111111</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:10">
       <c r="A43" s="20">
         <v>46121</v>
       </c>
@@ -3103,7 +3103,7 @@
         <v>0.49513888888888891</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:10">
       <c r="A44" s="20">
         <v>46121</v>
       </c>
@@ -3134,7 +3134,7 @@
         <v>0.52083333333333337</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:10">
       <c r="A45" s="20">
         <v>46121</v>
       </c>
@@ -3165,7 +3165,7 @@
         <v>0.66319444444444442</v>
       </c>
     </row>
-    <row r="46" spans="1:10" ht="25.2" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:10" ht="25.15">
       <c r="A46" s="20">
         <v>46121</v>
       </c>
@@ -3196,7 +3196,7 @@
         <v>0.71875</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:10">
       <c r="A47" s="20">
         <v>46122</v>
       </c>
@@ -3227,7 +3227,7 @@
         <v>0.33819444444444446</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:10">
       <c r="A48" s="20">
         <v>46122</v>
       </c>
@@ -3258,7 +3258,7 @@
         <v>0.4548611111111111</v>
       </c>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:10">
       <c r="A49" s="20">
         <v>46122</v>
       </c>
@@ -3289,7 +3289,7 @@
         <v>0.4909722222222222</v>
       </c>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:10">
       <c r="A50" s="20">
         <v>46122</v>
       </c>
@@ -3320,7 +3320,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:10">
       <c r="A51" s="20">
         <v>46122</v>
       </c>
@@ -3351,7 +3351,7 @@
         <v>0.625</v>
       </c>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:10">
       <c r="A52" s="29">
         <v>46123</v>
       </c>
@@ -3370,7 +3370,7 @@
       <c r="I52" s="33"/>
       <c r="J52" s="33"/>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:10">
       <c r="A53" s="29">
         <v>46124</v>
       </c>
@@ -3389,7 +3389,7 @@
       <c r="I53" s="33"/>
       <c r="J53" s="33"/>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:10">
       <c r="A54" s="20">
         <v>46125</v>
       </c>
@@ -3420,7 +3420,7 @@
         <v>0.34097222222222223</v>
       </c>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:10">
       <c r="A55" s="20">
         <v>46125</v>
       </c>
@@ -3451,7 +3451,7 @@
         <v>0.4548611111111111</v>
       </c>
     </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:10">
       <c r="A56" s="20">
         <v>46125</v>
       </c>
@@ -3482,7 +3482,7 @@
         <v>0.48055555555555557</v>
       </c>
     </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:10">
       <c r="A57" s="20">
         <v>46125</v>
       </c>
@@ -3513,7 +3513,7 @@
         <v>0.54027777777777775</v>
       </c>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:10">
       <c r="A58" s="20">
         <v>46125</v>
       </c>
@@ -3544,7 +3544,7 @@
         <v>0.66319444444444442</v>
       </c>
     </row>
-    <row r="59" spans="1:10" ht="25.2" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:10" ht="25.15">
       <c r="A59" s="20">
         <v>46125</v>
       </c>
@@ -3575,7 +3575,7 @@
         <v>0.70972222222222225</v>
       </c>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:10">
       <c r="A60" s="20">
         <v>46126</v>
       </c>
@@ -3606,7 +3606,7 @@
         <v>0.33888888888888891</v>
       </c>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:10">
       <c r="A61" s="20">
         <v>46126</v>
       </c>
@@ -3637,7 +3637,7 @@
         <v>0.4548611111111111</v>
       </c>
     </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:10">
       <c r="A62" s="20">
         <v>46126</v>
       </c>
@@ -3668,7 +3668,7 @@
         <v>0.49305555555555558</v>
       </c>
     </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:10">
       <c r="A63" s="20">
         <v>46126</v>
       </c>
@@ -3699,7 +3699,7 @@
         <v>0.52430555555555558</v>
       </c>
     </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:10">
       <c r="A64" s="20">
         <v>46126</v>
       </c>
@@ -3730,7 +3730,7 @@
         <v>0.54166666666666663</v>
       </c>
     </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:10">
       <c r="A65" s="20">
         <v>46126</v>
       </c>
@@ -3761,7 +3761,7 @@
         <v>0.66319444444444442</v>
       </c>
     </row>
-    <row r="66" spans="1:10" ht="25.2" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:10" ht="25.15">
       <c r="A66" s="20">
         <v>46126</v>
       </c>
@@ -3792,7 +3792,7 @@
         <v>0.70486111111111116</v>
       </c>
     </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:10">
       <c r="A67" s="20">
         <v>46126</v>
       </c>
@@ -3823,7 +3823,7 @@
         <v>0.72222222222222221</v>
       </c>
     </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:10">
       <c r="A68" s="20">
         <v>46127</v>
       </c>
@@ -3854,7 +3854,7 @@
         <v>0.33611111111111114</v>
       </c>
     </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:10">
       <c r="A69" s="20">
         <v>46127</v>
       </c>
@@ -3885,7 +3885,7 @@
         <v>0.4548611111111111</v>
       </c>
     </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:10">
       <c r="A70" s="20">
         <v>46127</v>
       </c>
@@ -3916,7 +3916,7 @@
         <v>0.47916666666666669</v>
       </c>
     </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:10">
       <c r="A71" s="20">
         <v>46127</v>
       </c>
@@ -3947,7 +3947,7 @@
         <v>0.53125</v>
       </c>
     </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:10">
       <c r="A72" s="20">
         <v>46127</v>
       </c>
@@ -3978,7 +3978,7 @@
         <v>0.66319444444444442</v>
       </c>
     </row>
-    <row r="73" spans="1:10" ht="25.2" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:10" ht="25.15">
       <c r="A73" s="20">
         <v>46127</v>
       </c>
@@ -4009,7 +4009,7 @@
         <v>0.72291666666666665</v>
       </c>
     </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:10">
       <c r="A74" s="20">
         <v>46128</v>
       </c>
@@ -4040,7 +4040,7 @@
         <v>0.33819444444444446</v>
       </c>
     </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:10">
       <c r="A75" s="20">
         <v>46128</v>
       </c>
@@ -4071,7 +4071,7 @@
         <v>0.4548611111111111</v>
       </c>
     </row>
-    <row r="76" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:10">
       <c r="A76" s="20">
         <v>46128</v>
       </c>
@@ -4102,7 +4102,7 @@
         <v>0.48472222222222222</v>
       </c>
     </row>
-    <row r="77" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:10">
       <c r="A77" s="20">
         <v>46128</v>
       </c>
@@ -4133,7 +4133,7 @@
         <v>0.54166666666666663</v>
       </c>
     </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:10">
       <c r="A78" s="20">
         <v>46128</v>
       </c>
@@ -4164,7 +4164,7 @@
         <v>0.66319444444444442</v>
       </c>
     </row>
-    <row r="79" spans="1:10" ht="25.2" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:10" ht="25.15">
       <c r="A79" s="20">
         <v>46128</v>
       </c>
@@ -4195,7 +4195,7 @@
         <v>0.73263888888888884</v>
       </c>
     </row>
-    <row r="80" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:10">
       <c r="A80" s="20">
         <v>46129</v>
       </c>
@@ -4226,7 +4226,7 @@
         <v>0.36249999999999999</v>
       </c>
     </row>
-    <row r="81" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:10">
       <c r="A81" s="20">
         <v>46129</v>
       </c>
@@ -4257,7 +4257,7 @@
         <v>0.4548611111111111</v>
       </c>
     </row>
-    <row r="82" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:10">
       <c r="A82" s="20">
         <v>46129</v>
       </c>
@@ -4288,7 +4288,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="83" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:10">
       <c r="A83" s="20">
         <v>46129</v>
       </c>
@@ -4319,7 +4319,7 @@
         <v>0.53125</v>
       </c>
     </row>
-    <row r="84" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:10">
       <c r="A84" s="20">
         <v>46129</v>
       </c>
@@ -4350,7 +4350,7 @@
         <v>0.66319444444444442</v>
       </c>
     </row>
-    <row r="85" spans="1:10" ht="25.2" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:10" ht="25.15">
       <c r="A85" s="20">
         <v>46129</v>
       </c>
@@ -4381,7 +4381,7 @@
         <v>0.73263888888888884</v>
       </c>
     </row>
-    <row r="86" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:10">
       <c r="A86" s="29">
         <v>46130</v>
       </c>
@@ -4400,7 +4400,7 @@
       <c r="I86" s="33"/>
       <c r="J86" s="33"/>
     </row>
-    <row r="87" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:10">
       <c r="A87" s="29">
         <v>46131</v>
       </c>
@@ -4419,7 +4419,7 @@
       <c r="I87" s="33"/>
       <c r="J87" s="33"/>
     </row>
-    <row r="88" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:10">
       <c r="A88" s="20">
         <v>46132</v>
       </c>
@@ -4450,7 +4450,7 @@
         <v>0.34375</v>
       </c>
     </row>
-    <row r="89" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:10">
       <c r="A89" s="20">
         <v>46132</v>
       </c>
@@ -4481,7 +4481,7 @@
         <v>0.34652777777777777</v>
       </c>
     </row>
-    <row r="90" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:10">
       <c r="A90" s="20">
         <v>46132</v>
       </c>
@@ -4512,7 +4512,7 @@
         <v>0.4548611111111111</v>
       </c>
     </row>
-    <row r="91" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:10">
       <c r="A91" s="20">
         <v>46132</v>
       </c>
@@ -4543,7 +4543,7 @@
         <v>0.45833333333333331</v>
       </c>
     </row>
-    <row r="92" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:10">
       <c r="A92" s="20">
         <v>46132</v>
       </c>
@@ -4574,7 +4574,7 @@
         <v>0.53472222222222221</v>
       </c>
     </row>
-    <row r="93" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:10">
       <c r="A93" s="20">
         <v>46132</v>
       </c>
@@ -4605,7 +4605,7 @@
         <v>0.66319444444444442</v>
       </c>
     </row>
-    <row r="94" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:10">
       <c r="A94" s="20">
         <v>46132</v>
       </c>
@@ -4636,7 +4636,7 @@
         <v>0.69374999999999998</v>
       </c>
     </row>
-    <row r="95" spans="1:10" ht="25.2" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:10" ht="25.15">
       <c r="A95" s="20">
         <v>46132</v>
       </c>
@@ -4667,7 +4667,7 @@
         <v>0.71736111111111112</v>
       </c>
     </row>
-    <row r="96" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:10">
       <c r="A96" s="20">
         <v>46133</v>
       </c>
@@ -4698,7 +4698,7 @@
         <v>0.3347222222222222</v>
       </c>
     </row>
-    <row r="97" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:10">
       <c r="A97" s="20">
         <v>46133</v>
       </c>
@@ -4729,7 +4729,7 @@
         <v>0.4548611111111111</v>
       </c>
     </row>
-    <row r="98" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:10">
       <c r="A98" s="20">
         <v>46133</v>
       </c>
@@ -4760,7 +4760,7 @@
         <v>0.49791666666666667</v>
       </c>
     </row>
-    <row r="99" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:10">
       <c r="A99" s="20">
         <v>46133</v>
       </c>
@@ -4791,7 +4791,7 @@
         <v>0.53472222222222221</v>
       </c>
     </row>
-    <row r="100" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:10">
       <c r="A100" s="20">
         <v>46133</v>
       </c>
@@ -4822,7 +4822,7 @@
         <v>0.66319444444444442</v>
       </c>
     </row>
-    <row r="101" spans="1:10" ht="25.2" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:10" ht="25.15">
       <c r="A101" s="20">
         <v>46133</v>
       </c>
@@ -4853,7 +4853,7 @@
         <v>0.71180555555555558</v>
       </c>
     </row>
-    <row r="102" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:10">
       <c r="A102" s="20">
         <v>46134</v>
       </c>
@@ -4884,7 +4884,7 @@
         <v>0.33958333333333335</v>
       </c>
     </row>
-    <row r="103" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:10">
       <c r="A103" s="20">
         <v>46134</v>
       </c>
@@ -4915,7 +4915,7 @@
         <v>0.4548611111111111</v>
       </c>
     </row>
-    <row r="104" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:10">
       <c r="A104" s="20">
         <v>46134</v>
       </c>
@@ -4946,7 +4946,7 @@
         <v>0.51041666666666663</v>
       </c>
     </row>
-    <row r="105" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:10">
       <c r="A105" s="20">
         <v>46134</v>
       </c>
@@ -4977,7 +4977,7 @@
         <v>0.53472222222222221</v>
       </c>
     </row>
-    <row r="106" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:10">
       <c r="A106" s="20">
         <v>46134</v>
       </c>
@@ -5008,7 +5008,7 @@
         <v>0.66319444444444442</v>
       </c>
     </row>
-    <row r="107" spans="1:10" ht="25.2" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:10" ht="25.15">
       <c r="A107" s="20">
         <v>46134</v>
       </c>
@@ -5039,7 +5039,7 @@
         <v>0.71527777777777779</v>
       </c>
     </row>
-    <row r="108" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:10">
       <c r="A108" s="20">
         <v>46134</v>
       </c>
@@ -5070,7 +5070,7 @@
         <v>0.74861111111111112</v>
       </c>
     </row>
-    <row r="109" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:10">
       <c r="A109" s="20">
         <v>46135</v>
       </c>
@@ -5101,7 +5101,7 @@
         <v>0.33611111111111114</v>
       </c>
     </row>
-    <row r="110" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:10">
       <c r="A110" s="20">
         <v>46135</v>
       </c>
@@ -5132,7 +5132,7 @@
         <v>0.4548611111111111</v>
       </c>
     </row>
-    <row r="111" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:10">
       <c r="A111" s="20">
         <v>46135</v>
       </c>
@@ -5163,7 +5163,7 @@
         <v>0.50763888888888886</v>
       </c>
     </row>
-    <row r="112" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:10">
       <c r="A112" s="20">
         <v>46135</v>
       </c>
@@ -5194,7 +5194,7 @@
         <v>0.52083333333333337</v>
       </c>
     </row>
-    <row r="113" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:10">
       <c r="A113" s="20">
         <v>46135</v>
       </c>
@@ -5225,7 +5225,7 @@
         <v>0.65972222222222221</v>
       </c>
     </row>
-    <row r="114" spans="1:10" ht="25.2" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:10" ht="25.15">
       <c r="A114" s="20">
         <v>46135</v>
       </c>
@@ -5256,7 +5256,7 @@
         <v>0.70694444444444449</v>
       </c>
     </row>
-    <row r="115" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:10">
       <c r="A115" s="20">
         <v>46136</v>
       </c>
@@ -5287,7 +5287,7 @@
         <v>0.34236111111111112</v>
       </c>
     </row>
-    <row r="116" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:10">
       <c r="A116" s="20">
         <v>46136</v>
       </c>
@@ -5318,7 +5318,7 @@
         <v>0.4548611111111111</v>
       </c>
     </row>
-    <row r="117" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:10">
       <c r="A117" s="20">
         <v>46136</v>
       </c>
@@ -5349,7 +5349,7 @@
         <v>0.49236111111111114</v>
       </c>
     </row>
-    <row r="118" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:10">
       <c r="A118" s="20">
         <v>46136</v>
       </c>
@@ -5380,7 +5380,7 @@
         <v>0.53472222222222221</v>
       </c>
     </row>
-    <row r="119" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:10">
       <c r="A119" s="20">
         <v>46136</v>
       </c>
@@ -5411,7 +5411,7 @@
         <v>0.60416666666666663</v>
       </c>
     </row>
-    <row r="120" spans="1:10" ht="25.2" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:10" ht="25.15">
       <c r="A120" s="20">
         <v>46136</v>
       </c>
@@ -5442,7 +5442,7 @@
         <v>0.61527777777777781</v>
       </c>
     </row>
-    <row r="121" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:10">
       <c r="A121" s="20">
         <v>46136</v>
       </c>
@@ -5473,7 +5473,7 @@
         <v>0.66319444444444442</v>
       </c>
     </row>
-    <row r="122" spans="1:10" ht="25.2" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:10" ht="25.15">
       <c r="A122" s="20">
         <v>46136</v>
       </c>
@@ -5504,7 +5504,7 @@
         <v>0.72916666666666663</v>
       </c>
     </row>
-    <row r="123" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:10">
       <c r="A123" s="29">
         <v>46137</v>
       </c>
@@ -5523,7 +5523,7 @@
       <c r="I123" s="33"/>
       <c r="J123" s="33"/>
     </row>
-    <row r="124" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:10">
       <c r="A124" s="29">
         <v>46138</v>
       </c>
@@ -5542,7 +5542,7 @@
       <c r="I124" s="33"/>
       <c r="J124" s="33"/>
     </row>
-    <row r="125" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:10">
       <c r="A125" s="43">
         <v>46139</v>
       </c>
@@ -5573,7 +5573,7 @@
         <v>0.66666666666666663</v>
       </c>
     </row>
-    <row r="126" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:10">
       <c r="A126" s="20">
         <v>46140</v>
       </c>
@@ -5604,7 +5604,7 @@
         <v>0.33750000000000002</v>
       </c>
     </row>
-    <row r="127" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:10">
       <c r="A127" s="20">
         <v>46140</v>
       </c>
@@ -5635,7 +5635,7 @@
         <v>0.4548611111111111</v>
       </c>
     </row>
-    <row r="128" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:10">
       <c r="A128" s="20">
         <v>46140</v>
       </c>
@@ -5666,7 +5666,7 @@
         <v>0.50138888888888888</v>
       </c>
     </row>
-    <row r="129" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:10">
       <c r="A129" s="20">
         <v>46140</v>
       </c>
@@ -5697,7 +5697,7 @@
         <v>0.53125</v>
       </c>
     </row>
-    <row r="130" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:10">
       <c r="A130" s="20">
         <v>46140</v>
       </c>
@@ -5728,7 +5728,7 @@
         <v>0.60416666666666663</v>
       </c>
     </row>
-    <row r="131" spans="1:10" ht="25.2" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:10" ht="25.15">
       <c r="A131" s="20">
         <v>46140</v>
       </c>
@@ -5759,7 +5759,7 @@
         <v>0.64722222222222225</v>
       </c>
     </row>
-    <row r="132" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:10">
       <c r="A132" s="20">
         <v>46140</v>
       </c>
@@ -5790,7 +5790,7 @@
         <v>0.66319444444444442</v>
       </c>
     </row>
-    <row r="133" spans="1:10" ht="25.2" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:10" ht="25.15">
       <c r="A133" s="20">
         <v>46140</v>
       </c>
@@ -5821,7 +5821,7 @@
         <v>0.70833333333333337</v>
       </c>
     </row>
-    <row r="134" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:10">
       <c r="A134" s="20">
         <v>46141</v>
       </c>
@@ -5852,7 +5852,7 @@
         <v>0.34652777777777777</v>
       </c>
     </row>
-    <row r="135" spans="1:10" ht="25.2" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:10" ht="25.15">
       <c r="A135" s="20">
         <v>46141</v>
       </c>
@@ -5883,7 +5883,7 @@
         <v>0.39583333333333331</v>
       </c>
     </row>
-    <row r="136" spans="1:10" ht="25.2" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:10" ht="25.15">
       <c r="A136" s="20">
         <v>46141</v>
       </c>
@@ -5914,7 +5914,7 @@
         <v>0.45347222222222222</v>
       </c>
     </row>
-    <row r="137" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:10">
       <c r="A137" s="20">
         <v>46141</v>
       </c>
@@ -5945,7 +5945,7 @@
         <v>0.49444444444444446</v>
       </c>
     </row>
-    <row r="138" spans="1:10" ht="25.2" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:10" ht="25.15">
       <c r="A138" s="20">
         <v>46141</v>
       </c>
@@ -5976,7 +5976,7 @@
         <v>0.53472222222222221</v>
       </c>
     </row>
-    <row r="139" spans="1:10" ht="25.2" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:10" ht="25.15">
       <c r="A139" s="20">
         <v>46141</v>
       </c>
@@ -6007,7 +6007,7 @@
         <v>0.66319444444444442</v>
       </c>
     </row>
-    <row r="140" spans="1:10" ht="25.2" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:10" ht="25.15">
       <c r="A140" s="20">
         <v>46141</v>
       </c>
@@ -6038,7 +6038,7 @@
         <v>0.71111111111111114</v>
       </c>
     </row>
-    <row r="141" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:10">
       <c r="A141" s="20">
         <v>46142</v>
       </c>
@@ -6069,7 +6069,7 @@
         <v>0.34791666666666665</v>
       </c>
     </row>
-    <row r="142" spans="1:10" ht="25.2" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:10" ht="25.15">
       <c r="A142" s="20">
         <v>46142</v>
       </c>
@@ -6100,7 +6100,7 @@
         <v>0.41666666666666669</v>
       </c>
     </row>
-    <row r="143" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:10">
       <c r="A143" s="20">
         <v>46142</v>
       </c>
@@ -6131,7 +6131,7 @@
         <v>0.45833333333333331</v>
       </c>
     </row>
-    <row r="144" spans="1:10" ht="25.2" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:10" ht="25.15">
       <c r="A144" s="20">
         <v>46142</v>
       </c>
@@ -6162,7 +6162,7 @@
         <v>0.53472222222222221</v>
       </c>
     </row>
-    <row r="145" spans="1:10" ht="25.2" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:10" ht="25.15">
       <c r="A145" s="20">
         <v>46142</v>
       </c>
@@ -6193,7 +6193,7 @@
         <v>0.60416666666666663</v>
       </c>
     </row>
-    <row r="146" spans="1:10" ht="25.2" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:10" ht="25.15">
       <c r="A146" s="20">
         <v>46142</v>
       </c>
@@ -6224,7 +6224,7 @@
         <v>0.66319444444444442</v>
       </c>
     </row>
-    <row r="147" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:10">
       <c r="A147" s="20">
         <v>46142</v>
       </c>
@@ -6255,7 +6255,7 @@
         <v>0.71597222222222223</v>
       </c>
     </row>
-    <row r="148" spans="1:10" ht="25.2" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:10" ht="25.15">
       <c r="A148" s="20">
         <v>46142</v>
       </c>
@@ -6286,7 +6286,7 @@
         <v>0.72222222222222221</v>
       </c>
     </row>
-    <row r="149" spans="1:10" ht="13.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:10" ht="13.9" customHeight="1" thickBot="1">
       <c r="A149" s="42"/>
       <c r="B149" s="42"/>
       <c r="G149" s="37"/>
@@ -6294,7 +6294,7 @@
       <c r="I149" s="61"/>
       <c r="J149" s="61"/>
     </row>
-    <row r="150" spans="1:10" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:10" ht="13.9" customHeight="1">
       <c r="A150" s="2"/>
       <c r="B150" s="2"/>
       <c r="C150" s="3"/>
@@ -6307,7 +6307,7 @@
       </c>
       <c r="H150" s="37"/>
     </row>
-    <row r="151" spans="1:10" ht="13.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:10" ht="13.9" customHeight="1" thickBot="1">
       <c r="A151" s="2"/>
       <c r="B151" s="2"/>
       <c r="C151" s="7"/>
@@ -6320,7 +6320,7 @@
       </c>
       <c r="H151" s="37"/>
     </row>
-    <row r="152" spans="1:10" ht="13.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:10" ht="13.9" customHeight="1" thickBot="1">
       <c r="A152" s="91" t="s">
         <v>43</v>
       </c>
@@ -6331,7 +6331,7 @@
       <c r="F152" s="1"/>
       <c r="H152" s="37"/>
     </row>
-    <row r="153" spans="1:10" ht="13.8" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:10" ht="13.9">
       <c r="A153" s="11"/>
       <c r="B153" s="11"/>
       <c r="C153" s="4"/>
@@ -6345,7 +6345,7 @@
       </c>
       <c r="H153" s="35"/>
     </row>
-    <row r="154" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:10" ht="15" customHeight="1" thickBot="1">
       <c r="A154" s="92" t="s">
         <v>45</v>
       </c>
@@ -6361,7 +6361,7 @@
       </c>
       <c r="H154" s="37"/>
     </row>
-    <row r="155" spans="1:10" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:10" ht="14.45" thickBot="1">
       <c r="A155" s="1"/>
       <c r="B155" s="1"/>
       <c r="C155" s="1"/>
@@ -6375,7 +6375,7 @@
       </c>
       <c r="H155" s="37"/>
     </row>
-    <row r="156" spans="1:10" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:10" ht="13.9" thickBot="1">
       <c r="A156" s="1"/>
       <c r="B156" s="1"/>
       <c r="C156" s="1"/>
@@ -6384,7 +6384,7 @@
       <c r="F156" s="1"/>
       <c r="H156" s="37"/>
     </row>
-    <row r="157" spans="1:10" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:10" ht="13.9" thickBot="1">
       <c r="A157" s="1"/>
       <c r="B157" s="1"/>
       <c r="C157" s="1"/>
@@ -6395,7 +6395,7 @@
       <c r="F157" s="19"/>
       <c r="H157" s="37"/>
     </row>
-    <row r="158" spans="1:10" ht="13.2" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:10" ht="13.15" thickBot="1">
       <c r="E158" s="36"/>
       <c r="H158" s="37"/>
     </row>
@@ -6406,56 +6406,56 @@
   </mergeCells>
   <phoneticPr fontId="10" type="noConversion"/>
   <conditionalFormatting sqref="A6:B6 D7:E7">
-    <cfRule type="containsText" dxfId="15" priority="12" operator="containsText" text="Religious Leave">
+    <cfRule type="containsText" dxfId="22" priority="12" operator="containsText" text="Religious Leave">
       <formula>NOT(ISERROR(SEARCH("Religious Leave",A6)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="14" priority="13" operator="containsText" text="Birthday Leave">
+    <cfRule type="containsText" dxfId="21" priority="13" operator="containsText" text="Birthday Leave">
       <formula>NOT(ISERROR(SEARCH("Birthday Leave",A6)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="13" priority="14" operator="containsText" text="Study Leave">
+    <cfRule type="containsText" dxfId="20" priority="14" operator="containsText" text="Study Leave">
       <formula>NOT(ISERROR(SEARCH("Study Leave",A6)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="12" priority="15" operator="containsText" text="Family Responsibility Leave">
+    <cfRule type="containsText" dxfId="19" priority="15" operator="containsText" text="Family Responsibility Leave">
       <formula>NOT(ISERROR(SEARCH("Family Responsibility Leave",A6)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="11" priority="16" operator="containsText" text="Sick Leave">
+    <cfRule type="containsText" dxfId="18" priority="16" operator="containsText" text="Sick Leave">
       <formula>NOT(ISERROR(SEARCH("Sick Leave",A6)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="10" priority="17" operator="containsText" text="Annual Leave">
+    <cfRule type="containsText" dxfId="17" priority="17" operator="containsText" text="Annual Leave">
       <formula>NOT(ISERROR(SEARCH("Annual Leave",A6)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="18" operator="equal">
+    <cfRule type="cellIs" dxfId="16" priority="18" operator="equal">
       <formula>"Public Holiday"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8:B158">
-    <cfRule type="containsText" dxfId="8" priority="1" operator="containsText" text="Saturday">
+    <cfRule type="containsText" dxfId="15" priority="1" operator="containsText" text="Saturday">
       <formula>NOT(ISERROR(SEARCH("Saturday",B8)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="7" priority="2" operator="containsText" text="Sunday">
+    <cfRule type="containsText" dxfId="14" priority="2" operator="containsText" text="Sunday">
       <formula>NOT(ISERROR(SEARCH("Sunday",B8)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D150:E150 D152:E154 E157">
-    <cfRule type="containsText" dxfId="6" priority="3" operator="containsText" text="Religious Leave">
+    <cfRule type="containsText" dxfId="13" priority="3" operator="containsText" text="Religious Leave">
       <formula>NOT(ISERROR(SEARCH("Religious Leave",D150)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="5" priority="4" operator="containsText" text="Birthday Leave">
+    <cfRule type="containsText" dxfId="12" priority="4" operator="containsText" text="Birthday Leave">
       <formula>NOT(ISERROR(SEARCH("Birthday Leave",D150)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="4" priority="5" operator="containsText" text="Study Leave">
+    <cfRule type="containsText" dxfId="11" priority="5" operator="containsText" text="Study Leave">
       <formula>NOT(ISERROR(SEARCH("Study Leave",D150)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="3" priority="6" operator="containsText" text="Family Responsibility Leave">
+    <cfRule type="containsText" dxfId="10" priority="6" operator="containsText" text="Family Responsibility Leave">
       <formula>NOT(ISERROR(SEARCH("Family Responsibility Leave",D150)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="7" operator="containsText" text="Sick Leave">
+    <cfRule type="containsText" dxfId="9" priority="7" operator="containsText" text="Sick Leave">
       <formula>NOT(ISERROR(SEARCH("Sick Leave",D150)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="1" priority="8" operator="containsText" text="Annual Leave">
+    <cfRule type="containsText" dxfId="8" priority="8" operator="containsText" text="Annual Leave">
       <formula>NOT(ISERROR(SEARCH("Annual Leave",D150)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="9" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="9" operator="equal">
       <formula>"Public Holiday"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6507,18 +6507,18 @@
     <tabColor theme="4"/>
   </sheetPr>
   <dimension ref="B2:J76"/>
-  <sheetFormatPr defaultColWidth="8.69921875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.75" defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="8.69921875" style="48"/>
+    <col min="1" max="1" width="8.75" style="48"/>
     <col min="2" max="2" width="25.5" style="48" customWidth="1"/>
-    <col min="3" max="3" width="8.69921875" style="48"/>
-    <col min="4" max="4" width="19.19921875" style="48" customWidth="1"/>
-    <col min="5" max="5" width="8.69921875" style="48"/>
-    <col min="6" max="6" width="21.69921875" style="48" customWidth="1"/>
-    <col min="7" max="16384" width="8.69921875" style="48"/>
+    <col min="3" max="3" width="8.75" style="48"/>
+    <col min="4" max="4" width="19.25" style="48" customWidth="1"/>
+    <col min="5" max="5" width="8.75" style="48"/>
+    <col min="6" max="6" width="21.75" style="48" customWidth="1"/>
+    <col min="7" max="16384" width="8.75" style="48"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:10" ht="15" thickBot="1">
       <c r="B2" s="62" t="s">
         <v>14</v>
       </c>
@@ -6535,7 +6535,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="3" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:10">
       <c r="B3" s="62" t="s">
         <v>52</v>
       </c>
@@ -6553,7 +6553,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:10">
       <c r="B4" s="62" t="s">
         <v>56</v>
       </c>
@@ -6571,7 +6571,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:10">
       <c r="B5" s="62" t="s">
         <v>60</v>
       </c>
@@ -6586,7 +6586,7 @@
       </c>
       <c r="I5" s="70"/>
     </row>
-    <row r="6" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:10">
       <c r="B6" s="62" t="s">
         <v>64</v>
       </c>
@@ -6601,7 +6601,7 @@
       </c>
       <c r="I6" s="71"/>
     </row>
-    <row r="7" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:10">
       <c r="B7" s="62" t="s">
         <v>68</v>
       </c>
@@ -6616,7 +6616,7 @@
       </c>
       <c r="I7" s="72"/>
     </row>
-    <row r="8" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:10">
       <c r="B8" s="62" t="s">
         <v>72</v>
       </c>
@@ -6634,7 +6634,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="9" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:10">
       <c r="B9" s="62" t="s">
         <v>77</v>
       </c>
@@ -6652,7 +6652,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="10" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:10">
       <c r="B10" s="62" t="s">
         <v>82</v>
       </c>
@@ -6667,7 +6667,7 @@
       </c>
       <c r="I10" s="72"/>
     </row>
-    <row r="11" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:10">
       <c r="B11" s="62" t="s">
         <v>85</v>
       </c>
@@ -6685,7 +6685,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="12" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:10">
       <c r="B12" s="62" t="s">
         <v>90</v>
       </c>
@@ -6700,7 +6700,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="13" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:10">
       <c r="B13" s="62" t="s">
         <v>94</v>
       </c>
@@ -6712,7 +6712,7 @@
       </c>
       <c r="I13" s="73"/>
     </row>
-    <row r="14" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:10">
       <c r="B14" s="62" t="s">
         <v>97</v>
       </c>
@@ -6725,7 +6725,7 @@
       </c>
       <c r="I14" s="74"/>
     </row>
-    <row r="15" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:10">
       <c r="B15" s="62" t="s">
         <v>100</v>
       </c>
@@ -6738,7 +6738,7 @@
       </c>
       <c r="I15" s="73"/>
     </row>
-    <row r="16" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:10">
       <c r="B16" s="62" t="s">
         <v>103</v>
       </c>
@@ -6751,7 +6751,7 @@
       </c>
       <c r="I16" s="75"/>
     </row>
-    <row r="17" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:9">
       <c r="B17" s="62" t="s">
         <v>106</v>
       </c>
@@ -6764,7 +6764,7 @@
       </c>
       <c r="I17" s="73"/>
     </row>
-    <row r="18" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:9">
       <c r="B18" s="62" t="s">
         <v>109</v>
       </c>
@@ -6777,7 +6777,7 @@
       </c>
       <c r="I18" s="75"/>
     </row>
-    <row r="19" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:9">
       <c r="B19" s="62" t="s">
         <v>112</v>
       </c>
@@ -6790,7 +6790,7 @@
       </c>
       <c r="I19" s="76"/>
     </row>
-    <row r="20" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:9">
       <c r="B20" s="62" t="s">
         <v>114</v>
       </c>
@@ -6803,7 +6803,7 @@
       </c>
       <c r="I20" s="74"/>
     </row>
-    <row r="21" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:9">
       <c r="B21" s="62" t="s">
         <v>117</v>
       </c>
@@ -6816,7 +6816,7 @@
       </c>
       <c r="I21" s="72"/>
     </row>
-    <row r="22" spans="2:9" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:9" ht="27.6">
       <c r="B22" s="62" t="s">
         <v>120</v>
       </c>
@@ -6829,7 +6829,7 @@
       </c>
       <c r="I22" s="77"/>
     </row>
-    <row r="23" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:9">
       <c r="B23" s="62" t="s">
         <v>122</v>
       </c>
@@ -6842,7 +6842,7 @@
       </c>
       <c r="I23" s="78"/>
     </row>
-    <row r="24" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:9">
       <c r="B24" s="62" t="s">
         <v>125</v>
       </c>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="I24" s="79"/>
     </row>
-    <row r="25" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:9">
       <c r="B25" s="62" t="s">
         <v>127</v>
       </c>
@@ -6868,7 +6868,7 @@
       </c>
       <c r="I25" s="80"/>
     </row>
-    <row r="26" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:9">
       <c r="B26" s="62" t="s">
         <v>130</v>
       </c>
@@ -6879,7 +6879,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="27" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:9">
       <c r="B27" s="62" t="s">
         <v>133</v>
       </c>
@@ -6892,7 +6892,7 @@
       </c>
       <c r="I27" s="78"/>
     </row>
-    <row r="28" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:9">
       <c r="B28" s="62" t="s">
         <v>136</v>
       </c>
@@ -6905,7 +6905,7 @@
       </c>
       <c r="I28" s="66"/>
     </row>
-    <row r="29" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:9">
       <c r="B29" s="62" t="s">
         <v>139</v>
       </c>
@@ -6917,7 +6917,7 @@
       </c>
       <c r="I29" s="81"/>
     </row>
-    <row r="30" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:9">
       <c r="B30" s="62" t="s">
         <v>142</v>
       </c>
@@ -6929,7 +6929,7 @@
       </c>
       <c r="I30" s="79"/>
     </row>
-    <row r="31" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:9">
       <c r="B31" s="62" t="s">
         <v>145</v>
       </c>
@@ -6940,7 +6940,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="32" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:9">
       <c r="B32" s="62" t="s">
         <v>148</v>
       </c>
@@ -6952,7 +6952,7 @@
       </c>
       <c r="I32" s="80"/>
     </row>
-    <row r="33" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:9">
       <c r="B33" s="62" t="s">
         <v>151</v>
       </c>
@@ -6964,7 +6964,7 @@
       </c>
       <c r="I33" s="80"/>
     </row>
-    <row r="34" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:9">
       <c r="B34" s="62" t="s">
         <v>154</v>
       </c>
@@ -6976,7 +6976,7 @@
       </c>
       <c r="I34" s="65"/>
     </row>
-    <row r="35" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:9">
       <c r="B35" s="62" t="s">
         <v>157</v>
       </c>
@@ -6988,7 +6988,7 @@
       </c>
       <c r="I35" s="79"/>
     </row>
-    <row r="36" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:9">
       <c r="B36" s="62" t="s">
         <v>160</v>
       </c>
@@ -7000,7 +7000,7 @@
       </c>
       <c r="I36" s="72"/>
     </row>
-    <row r="37" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:9">
       <c r="B37" s="62" t="s">
         <v>163</v>
       </c>
@@ -7012,7 +7012,7 @@
       </c>
       <c r="I37" s="80"/>
     </row>
-    <row r="38" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:9">
       <c r="B38" s="62" t="s">
         <v>166</v>
       </c>
@@ -7024,7 +7024,7 @@
       </c>
       <c r="I38" s="79"/>
     </row>
-    <row r="39" spans="2:9" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:9" ht="27.6">
       <c r="B39" s="62" t="s">
         <v>168</v>
       </c>
@@ -7036,7 +7036,7 @@
       </c>
       <c r="I39" s="81"/>
     </row>
-    <row r="40" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:9">
       <c r="B40" s="62" t="s">
         <v>171</v>
       </c>
@@ -7048,7 +7048,7 @@
       </c>
       <c r="I40" s="82"/>
     </row>
-    <row r="41" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:9">
       <c r="B41" s="62" t="s">
         <v>174</v>
       </c>
@@ -7058,7 +7058,7 @@
       </c>
       <c r="I41" s="82"/>
     </row>
-    <row r="42" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:9">
       <c r="B42" s="62" t="s">
         <v>176</v>
       </c>
@@ -7067,7 +7067,7 @@
       </c>
       <c r="I42" s="79"/>
     </row>
-    <row r="43" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:9">
       <c r="B43" s="62" t="s">
         <v>178</v>
       </c>
@@ -7076,7 +7076,7 @@
       </c>
       <c r="I43" s="81"/>
     </row>
-    <row r="44" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:9">
       <c r="B44" s="90" t="s">
         <v>180</v>
       </c>
@@ -7084,158 +7084,158 @@
         <v>181</v>
       </c>
     </row>
-    <row r="45" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:9">
       <c r="H45" s="82" t="s">
         <v>182</v>
       </c>
       <c r="I45" s="80"/>
     </row>
-    <row r="46" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:9">
       <c r="H46" s="66" t="s">
         <v>183</v>
       </c>
       <c r="I46" s="83"/>
     </row>
-    <row r="47" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:9">
       <c r="B47" s="58"/>
       <c r="H47" s="82" t="s">
         <v>184</v>
       </c>
       <c r="I47" s="82"/>
     </row>
-    <row r="48" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:9">
       <c r="H48" s="66" t="s">
         <v>185</v>
       </c>
       <c r="I48" s="82"/>
     </row>
-    <row r="49" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="49" spans="8:9">
       <c r="H49" s="79" t="s">
         <v>186</v>
       </c>
       <c r="I49" s="82"/>
     </row>
-    <row r="50" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="50" spans="8:9">
       <c r="H50" s="66" t="s">
         <v>187</v>
       </c>
       <c r="I50" s="82"/>
     </row>
-    <row r="51" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="51" spans="8:9">
       <c r="H51" s="65" t="s">
         <v>188</v>
       </c>
       <c r="I51" s="82"/>
     </row>
-    <row r="52" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="52" spans="8:9">
       <c r="H52" s="82" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="53" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="53" spans="8:9">
       <c r="H53" s="79" t="s">
         <v>190</v>
       </c>
       <c r="I53" s="82"/>
     </row>
-    <row r="54" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="54" spans="8:9">
       <c r="H54" s="65" t="s">
         <v>191</v>
       </c>
       <c r="I54" s="81"/>
     </row>
-    <row r="55" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="55" spans="8:9">
       <c r="H55" s="66" t="s">
         <v>192</v>
       </c>
       <c r="I55" s="81"/>
     </row>
-    <row r="56" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="56" spans="8:9">
       <c r="H56" s="79" t="s">
         <v>193</v>
       </c>
       <c r="I56" s="66"/>
     </row>
-    <row r="57" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="57" spans="8:9">
       <c r="H57" s="66" t="s">
         <v>194</v>
       </c>
       <c r="I57" s="82"/>
     </row>
-    <row r="58" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="58" spans="8:9">
       <c r="H58" s="66" t="s">
         <v>195</v>
       </c>
       <c r="I58" s="82"/>
     </row>
-    <row r="59" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="59" spans="8:9">
       <c r="H59" s="82" t="s">
         <v>196</v>
       </c>
       <c r="I59" s="85"/>
     </row>
-    <row r="60" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="60" spans="8:9">
       <c r="H60" s="85" t="s">
         <v>197</v>
       </c>
       <c r="I60" s="65"/>
     </row>
-    <row r="61" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="61" spans="8:9">
       <c r="H61" s="65" t="s">
         <v>198</v>
       </c>
       <c r="I61" s="80"/>
     </row>
-    <row r="62" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="62" spans="8:9">
       <c r="H62" s="65" t="s">
         <v>199</v>
       </c>
       <c r="I62" s="65"/>
     </row>
-    <row r="63" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="63" spans="8:9">
       <c r="H63" s="80" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="64" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="64" spans="8:9">
       <c r="H64" s="89" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="65" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="65" spans="8:8">
       <c r="H65" s="81"/>
     </row>
-    <row r="66" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="66" spans="8:8">
       <c r="H66" s="79"/>
     </row>
-    <row r="67" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="67" spans="8:8">
       <c r="H67" s="82"/>
     </row>
-    <row r="68" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="68" spans="8:8">
       <c r="H68" s="72"/>
     </row>
-    <row r="69" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="69" spans="8:8">
       <c r="H69" s="82"/>
     </row>
-    <row r="70" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="70" spans="8:8">
       <c r="H70" s="66"/>
     </row>
-    <row r="71" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="71" spans="8:8">
       <c r="H71" s="79"/>
     </row>
-    <row r="72" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="72" spans="8:8">
       <c r="H72" s="81"/>
     </row>
-    <row r="73" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="73" spans="8:8">
       <c r="H73" s="70"/>
     </row>
-    <row r="74" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="74" spans="8:8">
       <c r="H74" s="77"/>
     </row>
-    <row r="75" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="75" spans="8:8">
       <c r="H75" s="86"/>
     </row>
-    <row r="76" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="76" spans="8:8">
       <c r="H76" s="86"/>
     </row>
   </sheetData>
@@ -7254,9 +7254,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -7398,47 +7401,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{16B8ED66-AEFF-4F41-B9B4-8B808B78E7B3}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AEC7E95B-D83C-4BF2-B258-C9BACBBE165C}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4EF9AF4E-B7EE-4998-83C5-0B5667258EA9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="606bf0c3-7c02-4ad1-9a2b-bad21eeec9a2"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4EF9AF4E-B7EE-4998-83C5-0B5667258EA9}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AEC7E95B-D83C-4BF2-B258-C9BACBBE165C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{16B8ED66-AEFF-4F41-B9B4-8B808B78E7B3}"/>
 </file>
 
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>